<commit_message>
fix: never overwrite calculated table columns with data
Shared _formulas.py decides which columns are calculated; openpyxl checks
formula columns before the data branch, and win32com writes only non-formula
column blocks (including .xlsb via cell formulas).
</commit_message>
<xml_diff>
--- a/tests/assets/test_template_readme_example.xlsx
+++ b/tests/assets/test_template_readme_example.xlsx
@@ -1366,9 +1366,7 @@
   <autoFilter ref="B10:E15" xr:uid="{7F7D5B32-EE89-457F-B88D-B7D28F74CF40}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{C79F06E1-AE75-4725-B0B2-E92B5ECE0FED}" name="Date" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{EA9C0E20-A10E-495F-B395-27ACE8D1620B}" name="Stock Price" dataDxfId="0">
-      <calculatedColumnFormula>100</calculatedColumnFormula>
-    </tableColumn>
+    <tableColumn id="2" xr3:uid="{EA9C0E20-A10E-495F-B395-27ACE8D1620B}" name="Stock Price" dataDxfId="0"/>
     <tableColumn id="4" xr3:uid="{BF5E6FDD-1F2E-40C2-9EED-AAA374E57C2C}" name="Target" dataDxfId="3">
       <calculatedColumnFormula>target_price</calculatedColumnFormula>
     </tableColumn>

</xml_diff>